<commit_message>
fix(artefacts): update product backlog avec nouvelles priorités
</commit_message>
<xml_diff>
--- a/docs/cadrage/equipe-24-product-backlog-v1.0.xlsx
+++ b/docs/cadrage/equipe-24-product-backlog-v1.0.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11122"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Meder\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gabriel/Documents/code/IPSSI_APOCAL_KIT/docs/cadrage/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6158EA70-6E3D-4C7B-BFB7-469FEA4789B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6EEE4587-E52A-0A4F-8772-030812AD9F89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17780" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Garde" sheetId="1" r:id="rId1"/>
@@ -679,9 +679,6 @@
     <t>25 user stories organisées en 7 epics, avec critères INVEST et MoSCoW</t>
   </si>
   <si>
-    <t>25 user stories : 6 MUST (MVP F1-F6) + 9 SHOULD R2 + 7 COULD R2 + 3 WON'T</t>
-  </si>
-  <si>
     <t>☑ Oui   ☐ Partiel   ☐ Non</t>
   </si>
   <si>
@@ -698,6 +695,9 @@
   </si>
   <si>
     <t>Cadrage</t>
+  </si>
+  <si>
+    <t>25 user stories : 8 MUST (MVP F1-F6 + EP-07 core) + 7 SHOULD</t>
   </si>
 </sst>
 </file>
@@ -717,158 +717,158 @@
       <sz val="72"/>
       <color rgb="FF1E1B4B"/>
       <name val="Cambria"/>
-      <charset val="1"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
       <sz val="14"/>
       <color rgb="FF1E1B4B"/>
       <name val="Cambria"/>
-      <charset val="1"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFF59E0B"/>
       <name val="Cambria"/>
-      <charset val="1"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
       <sz val="24"/>
       <color rgb="FF1E1B4B"/>
       <name val="Cambria"/>
-      <charset val="1"/>
+      <family val="1"/>
     </font>
     <font>
       <i/>
       <sz val="12"/>
       <color rgb="FF475569"/>
       <name val="Cambria"/>
-      <charset val="1"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF475569"/>
       <name val="Cambria"/>
-      <charset val="1"/>
+      <family val="1"/>
     </font>
     <font>
       <i/>
       <sz val="9"/>
       <color rgb="FF475569"/>
       <name val="Cambria"/>
-      <charset val="1"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color rgb="FFF59E0B"/>
       <name val="Cambria"/>
-      <charset val="1"/>
+      <family val="1"/>
     </font>
     <font>
       <i/>
       <sz val="10"/>
       <color rgb="FF475569"/>
       <name val="Cambria"/>
-      <charset val="1"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF1E1B4B"/>
       <name val="Cambria"/>
-      <charset val="1"/>
+      <family val="1"/>
     </font>
     <font>
       <i/>
       <sz val="11"/>
       <color rgb="FF475569"/>
       <name val="Cambria"/>
-      <charset val="1"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
       <color rgb="FFF59E0B"/>
       <name val="Cambria"/>
-      <charset val="1"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
       <sz val="18"/>
       <color rgb="FF1E1B4B"/>
       <name val="Cambria"/>
-      <charset val="1"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
       <name val="Cambria"/>
-      <charset val="1"/>
+      <family val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF1E1B4B"/>
       <name val="Cambria"/>
-      <charset val="1"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF16A34A"/>
       <name val="Cambria"/>
-      <charset val="1"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFDC2626"/>
       <name val="Cambria"/>
-      <charset val="1"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF1E1B4B"/>
       <name val="Cambria"/>
-      <charset val="1"/>
+      <family val="1"/>
     </font>
     <font>
       <sz val="9"/>
       <color rgb="FF1E1B4B"/>
       <name val="Cambria"/>
-      <charset val="1"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFB45309"/>
       <name val="Cambria"/>
-      <charset val="1"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FF475569"/>
       <name val="Cambria"/>
-      <charset val="1"/>
+      <family val="1"/>
     </font>
     <font>
       <b/>
       <sz val="14"/>
       <color rgb="FF16A34A"/>
       <name val="Cambria"/>
-      <charset val="1"/>
+      <family val="1"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF1E1B4B"/>
       <name val="Cambria"/>
-      <charset val="1"/>
+      <family val="1"/>
     </font>
     <font>
       <sz val="9"/>
@@ -1301,43 +1301,43 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:B21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4" customWidth="1"/>
     <col min="2" max="2" width="90" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2" ht="88.5" x14ac:dyDescent="1.1000000000000001">
+    <row r="2" spans="2:2" ht="89" x14ac:dyDescent="0.85">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="2:2" ht="18" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:2" ht="18" x14ac:dyDescent="0.2">
       <c r="B4" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B8" s="3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:2" ht="30" x14ac:dyDescent="0.4">
+    <row r="10" spans="2:2" ht="30" x14ac:dyDescent="0.3">
       <c r="B10" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="12" spans="2:2" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:2" ht="16" x14ac:dyDescent="0.2">
       <c r="B12" s="5" t="s">
         <v>207</v>
       </c>
     </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B20" s="6" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B21" s="7" t="s">
         <v>5</v>
       </c>
@@ -1351,24 +1351,24 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B2:C13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
     <col min="2" max="2" width="25" customWidth="1"/>
     <col min="3" max="3" width="106" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:3" ht="16" x14ac:dyDescent="0.2">
       <c r="B2" s="8" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B3" s="9" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="2:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B5" s="10" t="s">
         <v>8</v>
       </c>
@@ -1376,7 +1376,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="6" spans="2:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="10" t="s">
         <v>9</v>
       </c>
@@ -1384,23 +1384,23 @@
         <v>205</v>
       </c>
     </row>
-    <row r="7" spans="2:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="10" t="s">
         <v>10</v>
       </c>
       <c r="C7" s="34" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="8" spans="2:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="10" t="s">
         <v>11</v>
       </c>
       <c r="C8" s="34" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="9" spans="2:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="10" t="s">
         <v>12</v>
       </c>
@@ -1408,7 +1408,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="2:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="2:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="10" t="s">
         <v>14</v>
       </c>
@@ -1416,12 +1416,12 @@
         <v>206</v>
       </c>
     </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B12" s="12" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B13" s="7" t="s">
         <v>16</v>
       </c>
@@ -1435,7 +1435,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:E13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
@@ -1444,17 +1444,17 @@
     <col min="5" max="5" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="22.5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="23" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>19</v>
       </c>
@@ -1462,7 +1462,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" ht="30" x14ac:dyDescent="0.2">
       <c r="A6" s="14" t="s">
         <v>21</v>
       </c>
@@ -1479,7 +1479,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="15" t="s">
         <v>26</v>
       </c>
@@ -1496,7 +1496,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="15" t="s">
         <v>31</v>
       </c>
@@ -1513,7 +1513,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="15" t="s">
         <v>35</v>
       </c>
@@ -1530,7 +1530,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="15" t="s">
         <v>39</v>
       </c>
@@ -1547,7 +1547,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="15" t="s">
         <v>43</v>
       </c>
@@ -1564,7 +1564,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="15" t="s">
         <v>47</v>
       </c>
@@ -1581,7 +1581,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="15" t="s">
         <v>51</v>
       </c>
@@ -1607,7 +1607,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:K35"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="8" customWidth="1"/>
     <col min="3" max="3" width="38" customWidth="1"/>
@@ -1620,17 +1620,17 @@
     <col min="11" max="11" width="10" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="22.5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="23" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>19</v>
       </c>
@@ -1638,7 +1638,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A5" s="3" t="s">
         <v>57</v>
       </c>
@@ -1646,7 +1646,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A6" s="17" t="s">
         <v>59</v>
       </c>
@@ -1654,7 +1654,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A7" s="18" t="s">
         <v>61</v>
       </c>
@@ -1662,7 +1662,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="9" spans="1:11" ht="28.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" ht="30" x14ac:dyDescent="0.2">
       <c r="A9" s="14" t="s">
         <v>21</v>
       </c>
@@ -1697,7 +1697,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="19" t="s">
         <v>71</v>
       </c>
@@ -1732,7 +1732,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="11" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="19" t="s">
         <v>79</v>
       </c>
@@ -1767,7 +1767,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="12" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="19" t="s">
         <v>82</v>
       </c>
@@ -1802,7 +1802,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="13" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="19" t="s">
         <v>86</v>
       </c>
@@ -1837,7 +1837,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="19" t="s">
         <v>90</v>
       </c>
@@ -1872,7 +1872,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="19" t="s">
         <v>93</v>
       </c>
@@ -1907,7 +1907,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="19" t="s">
         <v>97</v>
       </c>
@@ -1936,13 +1936,13 @@
         <v>76</v>
       </c>
       <c r="J16" s="20" t="s">
-        <v>101</v>
+        <v>112</v>
       </c>
       <c r="K16" s="20" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="19" t="s">
         <v>103</v>
       </c>
@@ -1971,13 +1971,13 @@
         <v>76</v>
       </c>
       <c r="J17" s="20" t="s">
-        <v>101</v>
+        <v>30</v>
       </c>
       <c r="K17" s="20" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="19" t="s">
         <v>106</v>
       </c>
@@ -2006,13 +2006,13 @@
         <v>76</v>
       </c>
       <c r="J18" s="20" t="s">
-        <v>101</v>
+        <v>30</v>
       </c>
       <c r="K18" s="20" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="19" t="s">
         <v>109</v>
       </c>
@@ -2041,13 +2041,13 @@
         <v>76</v>
       </c>
       <c r="J19" s="20" t="s">
-        <v>112</v>
+        <v>30</v>
       </c>
       <c r="K19" s="20" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="20" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="19" t="s">
         <v>113</v>
       </c>
@@ -2082,7 +2082,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="21" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="19" t="s">
         <v>116</v>
       </c>
@@ -2117,7 +2117,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="22" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="19" t="s">
         <v>121</v>
       </c>
@@ -2152,7 +2152,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="19" t="s">
         <v>125</v>
       </c>
@@ -2187,7 +2187,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="24" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="19" t="s">
         <v>128</v>
       </c>
@@ -2222,7 +2222,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="25" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="19" t="s">
         <v>132</v>
       </c>
@@ -2257,7 +2257,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="26" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="19" t="s">
         <v>135</v>
       </c>
@@ -2292,7 +2292,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="27" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="19" t="s">
         <v>138</v>
       </c>
@@ -2308,9 +2308,7 @@
       <c r="E27" s="24" t="s">
         <v>141</v>
       </c>
-      <c r="F27" s="20">
-        <v>13</v>
-      </c>
+      <c r="F27" s="20"/>
       <c r="G27" s="20" t="s">
         <v>142</v>
       </c>
@@ -2327,7 +2325,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="28" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="19" t="s">
         <v>144</v>
       </c>
@@ -2343,9 +2341,7 @@
       <c r="E28" s="24" t="s">
         <v>141</v>
       </c>
-      <c r="F28" s="20">
-        <v>21</v>
-      </c>
+      <c r="F28" s="20"/>
       <c r="G28" s="20" t="s">
         <v>146</v>
       </c>
@@ -2362,7 +2358,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="29" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="19" t="s">
         <v>147</v>
       </c>
@@ -2378,9 +2374,7 @@
       <c r="E29" s="24" t="s">
         <v>141</v>
       </c>
-      <c r="F29" s="20">
-        <v>13</v>
-      </c>
+      <c r="F29" s="20"/>
       <c r="G29" s="20" t="s">
         <v>149</v>
       </c>
@@ -2397,7 +2391,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="30" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="19" t="s">
         <v>150</v>
       </c>
@@ -2411,7 +2405,7 @@
         <v>130</v>
       </c>
       <c r="E30" s="22" t="s">
-        <v>99</v>
+        <v>74</v>
       </c>
       <c r="F30" s="20">
         <v>5</v>
@@ -2426,13 +2420,13 @@
         <v>76</v>
       </c>
       <c r="J30" s="20" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="K30" s="20" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="31" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="19" t="s">
         <v>153</v>
       </c>
@@ -2446,7 +2440,7 @@
         <v>130</v>
       </c>
       <c r="E31" s="22" t="s">
-        <v>99</v>
+        <v>74</v>
       </c>
       <c r="F31" s="20">
         <v>5</v>
@@ -2461,13 +2455,13 @@
         <v>76</v>
       </c>
       <c r="J31" s="20" t="s">
-        <v>101</v>
+        <v>120</v>
       </c>
       <c r="K31" s="20" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="32" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="19" t="s">
         <v>156</v>
       </c>
@@ -2496,13 +2490,13 @@
         <v>76</v>
       </c>
       <c r="J32" s="20" t="s">
-        <v>112</v>
+        <v>101</v>
       </c>
       <c r="K32" s="20" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="33" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="19" t="s">
         <v>159</v>
       </c>
@@ -2531,13 +2525,13 @@
         <v>76</v>
       </c>
       <c r="J33" s="20" t="s">
-        <v>112</v>
+        <v>30</v>
       </c>
       <c r="K33" s="20" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="34" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" ht="69.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="19" t="s">
         <v>162</v>
       </c>
@@ -2566,13 +2560,13 @@
         <v>76</v>
       </c>
       <c r="J34" s="20" t="s">
-        <v>112</v>
+        <v>30</v>
       </c>
       <c r="K34" s="20" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A35" s="25" t="s">
         <v>165</v>
       </c>
@@ -2581,8 +2575,8 @@
       <c r="D35" s="26"/>
       <c r="E35" s="26"/>
       <c r="F35" s="25">
-        <f>SUM(F10:F34)</f>
-        <v>165</v>
+        <f>SUMIF(J10:J34,"&lt;&gt;n.c.",F10:F34)</f>
+        <v>56</v>
       </c>
       <c r="G35" s="27" t="s">
         <v>204</v>
@@ -2601,122 +2595,122 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:A28"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="95" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="22.5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" ht="23" x14ac:dyDescent="0.25">
       <c r="A1" s="13" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
         <v>167</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" ht="18" x14ac:dyDescent="0.2">
       <c r="A4" s="28" t="s">
         <v>168</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A5" s="9" t="s">
         <v>169</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A7" s="29" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" s="29" t="s">
         <v>171</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A9" s="29" t="s">
         <v>172</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A10" s="29" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A11" s="29" t="s">
         <v>174</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A12" s="29" t="s">
         <v>175</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A13" s="29" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" s="29" t="s">
         <v>177</v>
       </c>
     </row>
-    <row r="17" spans="1:1" ht="18" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" ht="18" x14ac:dyDescent="0.2">
       <c r="A17" s="28" t="s">
         <v>178</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A18" s="9" t="s">
         <v>179</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A20" s="29" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A21" s="29" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A22" s="29" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A23" s="29" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A24" s="29" t="s">
         <v>184</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A25" s="29" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A26" s="29" t="s">
         <v>186</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A27" s="29" t="s">
         <v>187</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A28" s="29" t="s">
         <v>188</v>
       </c>
@@ -2730,7 +2724,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A2:D15"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="2" customWidth="1"/>
     <col min="2" max="2" width="50" customWidth="1"/>
@@ -2738,17 +2732,17 @@
     <col min="4" max="4" width="40" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:4" ht="18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="18" x14ac:dyDescent="0.2">
       <c r="B2" s="2" t="s">
         <v>189</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="B3" s="9" t="s">
         <v>190</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" s="14"/>
       <c r="B5" s="14" t="s">
         <v>191</v>
@@ -2760,97 +2754,97 @@
         <v>193</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B6" s="30" t="s">
         <v>194</v>
       </c>
       <c r="C6" s="31" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D6" s="30" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B7" s="30" t="s">
         <v>195</v>
       </c>
       <c r="C7" s="31" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D7" s="30" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="30" t="s">
         <v>196</v>
       </c>
       <c r="C8" s="31" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D8" s="33"/>
     </row>
-    <row r="9" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B9" s="30" t="s">
         <v>197</v>
       </c>
       <c r="C9" s="31" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="D9" s="33"/>
     </row>
-    <row r="10" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B10" s="30" t="s">
         <v>198</v>
       </c>
       <c r="C10" s="31" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D10" s="33"/>
     </row>
-    <row r="11" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B11" s="30" t="s">
         <v>199</v>
       </c>
       <c r="C11" s="31" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D11" s="33"/>
     </row>
-    <row r="12" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B12" s="30" t="s">
         <v>200</v>
       </c>
       <c r="C12" s="31" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D12" s="33"/>
     </row>
-    <row r="13" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B13" s="30" t="s">
         <v>201</v>
       </c>
       <c r="C13" s="31" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D13" s="33"/>
     </row>
-    <row r="14" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B14" s="30" t="s">
         <v>202</v>
       </c>
       <c r="C14" s="31" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D14" s="33"/>
     </row>
-    <row r="15" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B15" s="30" t="s">
         <v>203</v>
       </c>
       <c r="C15" s="31" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="D15" s="30"/>
     </row>

</xml_diff>